<commit_message>
chore: clean up empty code change sections in the changes log
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hanee\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7e71a7f51efef439/Business/tripple/Digi Menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E20DFB34-EA02-4768-9D05-FCC7B6A75540}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{FD36F3A3-C0BD-4176-B664-92451A287DD8}"/>
   </bookViews>
@@ -884,7 +884,7 @@
         <v>27</v>
       </c>
       <c r="C28">
-        <v>1700</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Enhance menu layout and descriptions; update item categories and prices
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7e71a7f51efef439/Business/tripple/Digi Menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF75EE0C-A753-4D4A-9744-C58DFDE3B44D}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C68A0AF-76F1-441F-837C-B4D15A7E6BF7}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{FD36F3A3-C0BD-4176-B664-92451A287DD8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="71">
   <si>
     <t>Espresso</t>
   </si>
@@ -50,15 +50,6 @@
     <t>Cappachino</t>
   </si>
   <si>
-    <t>Ristado</t>
-  </si>
-  <si>
-    <t>Picolo</t>
-  </si>
-  <si>
-    <t>Mocha Frappe</t>
-  </si>
-  <si>
     <t>Hazelnut Latte</t>
   </si>
   <si>
@@ -89,12 +80,6 @@
     <t>Iced Latte</t>
   </si>
   <si>
-    <t>Latte Frappe</t>
-  </si>
-  <si>
-    <t>Icecream Frappe</t>
-  </si>
-  <si>
     <t>Iced Hazelnut Latte</t>
   </si>
   <si>
@@ -110,12 +95,6 @@
     <t>Iced Mocha Latte</t>
   </si>
   <si>
-    <t>Spanish Frappe</t>
-  </si>
-  <si>
-    <t>Pistachio Frappe</t>
-  </si>
-  <si>
     <t>After Eight</t>
   </si>
   <si>
@@ -140,18 +119,6 @@
     <t>Berry Cola</t>
   </si>
   <si>
-    <t>Classic Macha</t>
-  </si>
-  <si>
-    <t>Strawberry Macha</t>
-  </si>
-  <si>
-    <t>Coconut Macha</t>
-  </si>
-  <si>
-    <t>Signature Coffee Frappe</t>
-  </si>
-  <si>
     <t>Crème Brulee Frappe</t>
   </si>
   <si>
@@ -207,6 +174,81 @@
   </si>
   <si>
     <t>Brownie</t>
+  </si>
+  <si>
+    <t>Signature Vanilla Frappe</t>
+  </si>
+  <si>
+    <t>Signature Mocha Frappe</t>
+  </si>
+  <si>
+    <t>Signature Pista Frappe</t>
+  </si>
+  <si>
+    <t>Signature Strawberry Frappe</t>
+  </si>
+  <si>
+    <t>Mango Salsa</t>
+  </si>
+  <si>
+    <t>Fudge Mocha Frappe</t>
+  </si>
+  <si>
+    <t>Trippleberry Frappe</t>
+  </si>
+  <si>
+    <t>Matcha Frappe</t>
+  </si>
+  <si>
+    <t>Mixberry Smoothie</t>
+  </si>
+  <si>
+    <t>Mango Smoothie</t>
+  </si>
+  <si>
+    <t>Mango Matcha</t>
+  </si>
+  <si>
+    <t>Coconut Matcha</t>
+  </si>
+  <si>
+    <t>Strawberry Matcha</t>
+  </si>
+  <si>
+    <t>Classic Matcha</t>
+  </si>
+  <si>
+    <t>Apple Peach</t>
+  </si>
+  <si>
+    <t>Mojito</t>
+  </si>
+  <si>
+    <t>All Day</t>
+  </si>
+  <si>
+    <t>English Breakfast</t>
+  </si>
+  <si>
+    <t>Shakshouka</t>
+  </si>
+  <si>
+    <t>Beef Quesadilla</t>
+  </si>
+  <si>
+    <t>Croissant Egg Sandwich</t>
+  </si>
+  <si>
+    <t>Chicken Parmesan Sandwich</t>
+  </si>
+  <si>
+    <t>Beef Philly Steak Sandwich</t>
+  </si>
+  <si>
+    <t>French Toast</t>
+  </si>
+  <si>
+    <t>Butter Croissant</t>
   </si>
 </sst>
 </file>
@@ -587,27 +629,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C49F82-9CEF-4AC2-BDF7-287561CD6482}">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="1" max="1" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
@@ -618,21 +661,21 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
       <c r="C3">
-        <v>900</v>
+        <v>700</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>500</v>
@@ -640,7 +683,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -651,7 +694,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
@@ -662,109 +705,109 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="C7">
-        <v>450</v>
+        <v>800</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
       </c>
       <c r="C8">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9">
-        <v>800</v>
+        <v>850</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C10">
-        <v>700</v>
+        <v>800</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11">
-        <v>850</v>
+        <v>800</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C12">
-        <v>800</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C13">
-        <v>800</v>
+        <v>650</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14">
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15">
-        <v>650</v>
+        <v>900</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C16">
         <v>900</v>
@@ -772,54 +815,54 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C17">
-        <v>900</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C18">
-        <v>900</v>
+        <v>800</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="C19">
-        <v>1000</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="C20">
-        <v>800</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C21">
         <v>1200</v>
@@ -827,32 +870,32 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="C22">
-        <v>1000</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C23">
-        <v>1050</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="C24">
         <v>1200</v>
@@ -860,10 +903,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="C25">
         <v>1200</v>
@@ -871,10 +914,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C26">
         <v>1200</v>
@@ -882,32 +925,32 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="C27">
-        <v>900</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C28">
-        <v>1200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="C29">
         <v>1000</v>
@@ -915,21 +958,21 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C30">
-        <v>1000</v>
+        <v>900</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C31">
         <v>900</v>
@@ -937,10 +980,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C32">
         <v>900</v>
@@ -948,10 +991,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C33">
         <v>900</v>
@@ -959,21 +1002,21 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C34">
-        <v>900</v>
+        <v>750</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B35" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="C35">
         <v>600</v>
@@ -981,10 +1024,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="C36">
         <v>850</v>
@@ -992,10 +1035,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B37" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C37">
         <v>600</v>
@@ -1003,76 +1046,76 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="C38">
-        <v>600</v>
+        <v>850</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B39" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C39">
-        <v>750</v>
+        <v>600</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="C40">
-        <v>950</v>
+        <v>600</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="B41" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="C41">
-        <v>950</v>
+        <v>750</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C42">
-        <v>700</v>
+        <v>950</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C43">
-        <v>850</v>
+        <v>950</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B44" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="C44">
         <v>950</v>
@@ -1080,45 +1123,188 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B45" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C45">
-        <v>800</v>
+        <v>950</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B46" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C46">
-        <v>350</v>
+        <v>700</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B47" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C47">
-        <v>400</v>
+        <v>850</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B48" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" t="s">
         <v>56</v>
       </c>
-      <c r="C48">
+      <c r="C49">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B50" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B51" t="s">
+        <v>64</v>
+      </c>
+      <c r="C51">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" t="s">
+        <v>65</v>
+      </c>
+      <c r="C52">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B53" t="s">
+        <v>66</v>
+      </c>
+      <c r="C53">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B54" t="s">
+        <v>67</v>
+      </c>
+      <c r="C54">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C55">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B56" t="s">
+        <v>69</v>
+      </c>
+      <c r="C56">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B57" t="s">
+        <v>42</v>
+      </c>
+      <c r="C57">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B58" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B59" t="s">
+        <v>44</v>
+      </c>
+      <c r="C59">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B60" t="s">
+        <v>45</v>
+      </c>
+      <c r="C60">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B61" t="s">
+        <v>70</v>
+      </c>
+      <c r="C61">
         <v>300</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update mocktail and matcha prices; adjust item descriptions in menu
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7e71a7f51efef439/Business/tripple/Digi Menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C68A0AF-76F1-441F-837C-B4D15A7E6BF7}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B952C687-070A-4875-B28A-94FCA1D78666}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{FD36F3A3-C0BD-4176-B664-92451A287DD8}"/>
   </bookViews>
@@ -310,6 +310,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1008,7 +1012,7 @@
         <v>50</v>
       </c>
       <c r="C34">
-        <v>750</v>
+        <v>850</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
@@ -1016,10 +1020,10 @@
         <v>32</v>
       </c>
       <c r="B35" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="C35">
-        <v>600</v>
+        <v>850</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
@@ -1027,10 +1031,10 @@
         <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="C36">
-        <v>850</v>
+        <v>750</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -1038,10 +1042,10 @@
         <v>32</v>
       </c>
       <c r="B37" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C37">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
@@ -1049,10 +1053,10 @@
         <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C38">
-        <v>850</v>
+        <v>600</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
@@ -1071,7 +1075,7 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="C40">
         <v>600</v>
@@ -1082,10 +1086,10 @@
         <v>32</v>
       </c>
       <c r="B41" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C41">
-        <v>750</v>
+        <v>600</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
@@ -1137,10 +1141,10 @@
         <v>40</v>
       </c>
       <c r="B46" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C46">
-        <v>700</v>
+        <v>950</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
@@ -1148,7 +1152,7 @@
         <v>40</v>
       </c>
       <c r="B47" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C47">
         <v>850</v>
@@ -1159,10 +1163,10 @@
         <v>40</v>
       </c>
       <c r="B48" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C48">
-        <v>950</v>
+        <v>850</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -1170,10 +1174,10 @@
         <v>40</v>
       </c>
       <c r="B49" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C49">
-        <v>950</v>
+        <v>700</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update menu items: enhance descriptions and add new dishes
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7e71a7f51efef439/Business/tripple/Digi Menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B952C687-070A-4875-B28A-94FCA1D78666}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0507C9AC-CDE9-41D0-9E67-AAEDBF44CB95}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{FD36F3A3-C0BD-4176-B664-92451A287DD8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="72">
   <si>
     <t>Espresso</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>Butter Croissant</t>
+  </si>
+  <si>
+    <t>Description</t>
   </si>
 </sst>
 </file>
@@ -292,9 +295,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -633,15 +639,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C49F82-9CEF-4AC2-BDF7-287561CD6482}">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -649,667 +656,670 @@
         <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="C2">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2">
+        <v>391.304347826087</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="C3">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3">
+        <v>608.69565217391312</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4">
+        <v>434.78260869565219</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="C5">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5">
+        <v>565.21739130434787</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C6">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6">
+        <v>565.21739130434787</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
       </c>
-      <c r="C7">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7">
+        <v>695.6521739130435</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
       </c>
-      <c r="C8">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8">
+        <v>608.69565217391312</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
       </c>
-      <c r="C9">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9">
+        <v>739.13043478260875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
       </c>
-      <c r="C10">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10">
+        <v>695.6521739130435</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B11" t="s">
         <v>8</v>
       </c>
-      <c r="C11">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11">
+        <v>695.6521739130435</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C12">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12">
+        <v>434.78260869565219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13">
+        <v>565.21739130434787</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
       </c>
-      <c r="C14">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B15" t="s">
         <v>15</v>
       </c>
-      <c r="C15">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
-      <c r="C16">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D16">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B17" t="s">
         <v>18</v>
       </c>
-      <c r="C17">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17">
+        <v>869.56521739130437</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B18" t="s">
         <v>17</v>
       </c>
-      <c r="C18">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D18">
+        <v>695.6521739130435</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B19" t="s">
         <v>46</v>
       </c>
-      <c r="C19">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B20" t="s">
         <v>47</v>
       </c>
-      <c r="C20">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D20">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B21" t="s">
         <v>48</v>
       </c>
-      <c r="C21">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D21">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B22" t="s">
         <v>49</v>
       </c>
-      <c r="C22">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D22">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B23" t="s">
         <v>51</v>
       </c>
-      <c r="C23">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D23">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B24" t="s">
         <v>52</v>
       </c>
-      <c r="C24">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D24">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B25" t="s">
         <v>53</v>
       </c>
-      <c r="C25">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D25">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B26" t="s">
         <v>19</v>
       </c>
-      <c r="C26">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D26">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B27" t="s">
         <v>20</v>
       </c>
-      <c r="C27">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D27">
+        <v>1043.4782608695652</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B28" t="s">
         <v>21</v>
       </c>
-      <c r="C28">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D28">
+        <v>869.56521739130437</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B29" t="s">
         <v>27</v>
       </c>
-      <c r="C29">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D29">
+        <v>869.56521739130437</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B30" t="s">
         <v>35</v>
       </c>
-      <c r="C30">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D30">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B31" t="s">
         <v>36</v>
       </c>
-      <c r="C31">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D31">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B32" t="s">
         <v>37</v>
       </c>
-      <c r="C32">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D32">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B33" t="s">
         <v>38</v>
       </c>
-      <c r="C33">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D33">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B34" t="s">
         <v>50</v>
       </c>
-      <c r="C34">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D34">
+        <v>739.13043478260875</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B35" t="s">
         <v>23</v>
       </c>
-      <c r="C35">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D35">
+        <v>739.13043478260875</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B36" t="s">
         <v>26</v>
       </c>
-      <c r="C36">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D36">
+        <v>652.17391304347836</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B37" t="s">
         <v>60</v>
       </c>
-      <c r="C37">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D37">
+        <v>608.69565217391312</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B38" t="s">
         <v>25</v>
       </c>
-      <c r="C38">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D38">
+        <v>521.73913043478262</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B39" t="s">
         <v>24</v>
       </c>
-      <c r="C39">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D39">
+        <v>521.73913043478262</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B40" t="s">
         <v>61</v>
       </c>
-      <c r="C40">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D40">
+        <v>521.73913043478262</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B41" t="s">
         <v>22</v>
       </c>
-      <c r="C41">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D41">
+        <v>521.73913043478262</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B42" t="s">
         <v>33</v>
       </c>
-      <c r="C42">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D42">
+        <v>826.08695652173924</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B43" t="s">
         <v>34</v>
       </c>
-      <c r="C43">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D43">
+        <v>826.08695652173924</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B44" t="s">
         <v>54</v>
       </c>
-      <c r="C44">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D44">
+        <v>826.08695652173924</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B45" t="s">
         <v>55</v>
       </c>
-      <c r="C45">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D45">
+        <v>826.08695652173924</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B46" t="s">
         <v>57</v>
       </c>
-      <c r="C46">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D46">
+        <v>826.08695652173924</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B47" t="s">
         <v>56</v>
       </c>
-      <c r="C47">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D47">
+        <v>739.13043478260875</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B48" t="s">
         <v>58</v>
       </c>
-      <c r="C48">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D48">
+        <v>739.13043478260875</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B49" t="s">
         <v>59</v>
       </c>
-      <c r="C49">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D49">
+        <v>608.69565217391312</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B50" t="s">
         <v>63</v>
       </c>
-      <c r="C50">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D50">
+        <v>956.52173913043487</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B51" t="s">
         <v>64</v>
       </c>
-      <c r="C51">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D51">
+        <v>608.69565217391312</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B52" t="s">
         <v>65</v>
       </c>
-      <c r="C52">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D52">
+        <v>869.56521739130437</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B53" t="s">
         <v>66</v>
       </c>
-      <c r="C53">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D53">
+        <v>782.60869565217399</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B54" t="s">
         <v>67</v>
       </c>
-      <c r="C54">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D54">
+        <v>1086.9565217391305</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B55" t="s">
         <v>68</v>
       </c>
-      <c r="C55">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D55">
+        <v>1304.3478260869567</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B56" t="s">
         <v>69</v>
       </c>
-      <c r="C56">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D56">
+        <v>608.69565217391312</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B57" t="s">
         <v>42</v>
       </c>
-      <c r="C57">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D57">
+        <v>695.6521739130435</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B58" t="s">
         <v>43</v>
       </c>
-      <c r="C58">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D58">
+        <v>304.34782608695656</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B59" t="s">
         <v>44</v>
       </c>
-      <c r="C59">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D59">
+        <v>347.82608695652175</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B60" t="s">
         <v>45</v>
       </c>
-      <c r="C60">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D60">
+        <v>260.86956521739131</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B61" t="s">
         <v>70</v>
       </c>
-      <c r="C61">
-        <v>300</v>
+      <c r="D61">
+        <v>260.86956521739131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>